<commit_message>
M5.2-6 샘플 단가 통일 + dogfood 3절 교체
</commit_message>
<xml_diff>
--- a/examples/dogfood/sales-2026-09.xlsx
+++ b/examples/dogfood/sales-2026-09.xlsx
@@ -458,7 +458,7 @@
         <v>40</v>
       </c>
       <c r="D2" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="E2" t="n">
         <v>440000</v>
@@ -479,7 +479,7 @@
         <v>80</v>
       </c>
       <c r="D3" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="E3" t="n">
         <v>880000</v>
@@ -500,7 +500,7 @@
         <v>30</v>
       </c>
       <c r="D4" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="E4" t="n">
         <v>330000</v>
@@ -521,7 +521,7 @@
         <v>50</v>
       </c>
       <c r="D5" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="E5" t="n">
         <v>550000</v>

</xml_diff>